<commit_message>
White and Blue UI
</commit_message>
<xml_diff>
--- a/reports/onprem_kubeadm_oracle_sizing.xlsx
+++ b/reports/onprem_kubeadm_oracle_sizing.xlsx
@@ -13,10 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROD-3Yr" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROD-4Yr" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROD-5Yr" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DR" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRE-PROD" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIT" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRE-PROD" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIT" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -561,7 +559,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>On-Premise Infrastructure Metrics — HDFC — 09 Apr 2026</t>
+          <t>On-Premise Infrastructure Metrics — Apple FCU — 16 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -617,19 +615,19 @@
       </c>
       <c r="B4" s="7" t="n"/>
       <c r="C4" s="8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -647,19 +645,19 @@
       </c>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="11" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
@@ -670,19 +668,19 @@
       </c>
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="8" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>43</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -700,19 +698,19 @@
       </c>
       <c r="B9" s="10" t="n"/>
       <c r="C9" s="11" t="n">
-        <v>100</v>
+        <v>2100</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>110</v>
+        <v>2310</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>121</v>
+        <v>2541</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>133</v>
+        <v>2795</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>146</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
@@ -723,19 +721,19 @@
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="8" t="n">
-        <v>100</v>
+        <v>5900</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>110</v>
+        <v>6490</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>121</v>
+        <v>7139</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>133</v>
+        <v>7852</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>146</v>
+        <v>8638</v>
       </c>
     </row>
   </sheetData>
@@ -744,683 +742,6 @@
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:O22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="4" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
-    <col width="4" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>SIT Environment On Premise</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>S.N.</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>Services/Instances</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Nodes</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Instance Type</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-CPU cores</t>
-        </is>
-      </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-RAM</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-Storage (GB)</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-CPU cores</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-RAM
-(GB)</t>
-        </is>
-      </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-Storage
-(TB)</t>
-        </is>
-      </c>
-      <c r="M2" s="13" t="n"/>
-      <c r="N2" s="13" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="O2" s="13" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="B3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Kubeadm Cluster</t>
-        </is>
-      </c>
-      <c r="M3" s="14" t="n"/>
-      <c r="N3" s="14" t="n"/>
-      <c r="O3" s="14" t="n"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Bootstrap machine</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>Kubeadm vendor to confirm on sizing.</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I4" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J4" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="L4" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M4" s="16" t="n"/>
-      <c r="N4" s="16" t="inlineStr"/>
-      <c r="O4" s="16" t="n"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>Bastion Host</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="inlineStr"/>
-      <c r="G5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>256</v>
-      </c>
-      <c r="J5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M5" s="19" t="n"/>
-      <c r="N5" s="19" t="inlineStr"/>
-      <c r="O5" s="19" t="n"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Master Nodes</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr"/>
-      <c r="G6" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J6" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="L6" s="17" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="M6" s="16" t="n"/>
-      <c r="N6" s="16" t="inlineStr"/>
-      <c r="O6" s="16" t="n"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Linux Worker Nodes (BUSINESSNEXT)</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F7" s="19" t="inlineStr"/>
-      <c r="G7" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>256</v>
-      </c>
-      <c r="J7" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="L7" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M7" s="19" t="n"/>
-      <c r="N7" s="19" t="inlineStr"/>
-      <c r="O7" s="19" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Operational Services</t>
-        </is>
-      </c>
-      <c r="M8" s="14" t="n"/>
-      <c r="N8" s="14" t="n"/>
-      <c r="O8" s="14" t="n"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Infra Nodes (Grafana &amp; Prometheus, EFK, Redis)</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr"/>
-      <c r="G9" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J9" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="K9" s="16" t="n">
-        <v>64</v>
-      </c>
-      <c r="L9" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M9" s="16" t="n"/>
-      <c r="N9" s="16" t="inlineStr"/>
-      <c r="O9" s="16" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>NFS Storage</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr"/>
-      <c r="F10" s="19" t="inlineStr"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n">
-        <v>2792</v>
-      </c>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="20" t="n">
-        <v>2.7265625</v>
-      </c>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="19" t="inlineStr"/>
-      <c r="O10" s="19" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Oracle Database</t>
-        </is>
-      </c>
-      <c r="M11" s="14" t="n"/>
-      <c r="N11" s="14" t="n"/>
-      <c r="O11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>OEL/RHEL</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="H12" s="16" t="n">
-        <v>240</v>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="J12" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="K12" s="16" t="n">
-        <v>240</v>
-      </c>
-      <c r="L12" s="17" t="n">
-        <v>0.29296875</v>
-      </c>
-      <c r="M12" s="16" t="n"/>
-      <c r="N12" s="16" t="inlineStr"/>
-      <c r="O12" s="16" t="n"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>Oracle License</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="inlineStr"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="19" t="n"/>
-      <c r="L13" s="19" t="n"/>
-      <c r="M13" s="19" t="n"/>
-      <c r="N13" s="19" t="inlineStr"/>
-      <c r="O13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Storage: SAN</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>20K IOPS</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr"/>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="J14" s="16" t="n"/>
-      <c r="K14" s="16" t="n"/>
-      <c r="L14" s="17" t="n">
-        <v>0.48828125</v>
-      </c>
-      <c r="M14" s="16" t="n"/>
-      <c r="N14" s="16" t="inlineStr"/>
-      <c r="O14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="n"/>
-      <c r="N15" s="14" t="n"/>
-      <c r="O15" s="14" t="n"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>S3 Storage</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>To be consumed from main NFS storage</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>Will be based on the number of documents provided, Considering per document size per Service Request of 512KB Each.</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="17" t="n">
-        <v>0.48828125</v>
-      </c>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="16" t="inlineStr"/>
-      <c r="O16" s="16" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Infrastructure &amp; Monitoring</t>
-        </is>
-      </c>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="14" t="n"/>
-      <c r="O17" s="14" t="n"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>SSL</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>Provided by Bank</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr"/>
-      <c r="G18" s="19" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="19" t="n"/>
-      <c r="J18" s="19" t="n"/>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="19" t="n"/>
-      <c r="M18" s="19" t="n"/>
-      <c r="N18" s="19" t="inlineStr"/>
-      <c r="O18" s="19" t="n"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Image Registry</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>For Containers docker images</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n">
-        <v>1024</v>
-      </c>
-      <c r="J19" s="16" t="n"/>
-      <c r="K19" s="16" t="n"/>
-      <c r="L19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="inlineStr"/>
-      <c r="O19" s="16" t="n"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>Web Application Firewall (WAF)</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="19" t="inlineStr"/>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>As per banks security policy.</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="19" t="n"/>
-      <c r="N20" s="19" t="inlineStr"/>
-      <c r="O20" s="19" t="n"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Bastion Host</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="16" t="inlineStr"/>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>As per banks policy.</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="I21" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J21" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="L21" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="16" t="inlineStr"/>
-      <c r="O21" s="16" t="n"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Email Service</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>Two million mails/month</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="19" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
-      <c r="M22" s="19" t="n"/>
-      <c r="N22" s="19" t="inlineStr"/>
-      <c r="O22" s="19" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C15:O15"/>
-    <mergeCell ref="C11:O11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1670,7 +991,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -1688,13 +1009,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>128</v>
+        <v>288</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -1766,12 +1087,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3016</v>
+        <v>12096</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>2.9453125</v>
+        <v>11.8125</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -1807,19 +1128,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>240</v>
+        <v>488</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>480</v>
+        <v>976</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.5859375</v>
@@ -1873,12 +1194,12 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>100</v>
+        <v>2100</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.1953125</v>
+        <v>4.1015625</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
@@ -1970,19 +1291,19 @@
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>240</v>
+        <v>488</v>
       </c>
       <c r="I18" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J18" s="16" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K18" s="16" t="n">
-        <v>240</v>
+        <v>488</v>
       </c>
       <c r="L18" s="17" t="n">
         <v>0.29296875</v>
@@ -2036,12 +1357,12 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
       <c r="I20" s="16" t="n">
-        <v>100</v>
+        <v>2100</v>
       </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="17" t="n">
-        <v>0.09765625</v>
+        <v>2.05078125</v>
       </c>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="inlineStr"/>
@@ -2083,12 +1404,12 @@
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n">
-        <v>100</v>
+        <v>5900</v>
       </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="n"/>
       <c r="L22" s="17" t="n">
-        <v>0.09765625</v>
+        <v>5.76171875</v>
       </c>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="inlineStr"/>
@@ -2537,7 +1858,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -2555,13 +1876,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>128</v>
+        <v>288</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -2633,12 +1954,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3036</v>
+        <v>12896</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>2.96484375</v>
+        <v>12.59375</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -2674,19 +1995,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>264</v>
+        <v>536</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>528</v>
+        <v>1072</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.5859375</v>
@@ -2740,12 +2061,12 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>110</v>
+        <v>2310</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.21484375</v>
+        <v>4.51171875</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
@@ -2837,19 +2158,19 @@
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>264</v>
+        <v>536</v>
       </c>
       <c r="I18" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J18" s="16" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="K18" s="16" t="n">
-        <v>264</v>
+        <v>536</v>
       </c>
       <c r="L18" s="17" t="n">
         <v>0.29296875</v>
@@ -2903,12 +2224,12 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
       <c r="I20" s="16" t="n">
-        <v>110</v>
+        <v>2310</v>
       </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="17" t="n">
-        <v>0.10742188</v>
+        <v>2.25585938</v>
       </c>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="inlineStr"/>
@@ -2950,12 +2271,12 @@
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n">
-        <v>110</v>
+        <v>6490</v>
       </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="n"/>
       <c r="L22" s="17" t="n">
-        <v>0.10742188</v>
+        <v>6.33789062</v>
       </c>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="inlineStr"/>
@@ -3404,7 +2725,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -3422,13 +2743,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>128</v>
+        <v>288</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -3500,12 +2821,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3058</v>
+        <v>13776</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>2.98632812</v>
+        <v>13.453125</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -3541,19 +2862,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>288</v>
+        <v>584</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>576</v>
+        <v>1168</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.5859375</v>
@@ -3607,12 +2928,12 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>121</v>
+        <v>2541</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.23632812</v>
+        <v>4.96289062</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
@@ -3704,19 +3025,19 @@
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>288</v>
+        <v>584</v>
       </c>
       <c r="I18" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J18" s="16" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="K18" s="16" t="n">
-        <v>288</v>
+        <v>584</v>
       </c>
       <c r="L18" s="17" t="n">
         <v>0.29296875</v>
@@ -3770,12 +3091,12 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
       <c r="I20" s="16" t="n">
-        <v>121</v>
+        <v>2541</v>
       </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="17" t="n">
-        <v>0.11816406</v>
+        <v>2.48144531</v>
       </c>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="inlineStr"/>
@@ -3817,12 +3138,12 @@
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n">
-        <v>121</v>
+        <v>7139</v>
       </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="n"/>
       <c r="L22" s="17" t="n">
-        <v>0.11816406</v>
+        <v>6.97167969</v>
       </c>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="inlineStr"/>
@@ -4271,7 +3592,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -4289,13 +3610,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>128</v>
+        <v>320</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -4367,12 +3688,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3082</v>
+        <v>14999</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>3.00976562</v>
+        <v>14.64746094</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -4408,19 +3729,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>312</v>
+        <v>648</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>624</v>
+        <v>1296</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.5859375</v>
@@ -4474,12 +3795,12 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>133</v>
+        <v>2795</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.25976562</v>
+        <v>5.45898438</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
@@ -4571,19 +3892,19 @@
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>312</v>
+        <v>648</v>
       </c>
       <c r="I18" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J18" s="16" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="K18" s="16" t="n">
-        <v>312</v>
+        <v>648</v>
       </c>
       <c r="L18" s="17" t="n">
         <v>0.29296875</v>
@@ -4637,12 +3958,12 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
       <c r="I20" s="16" t="n">
-        <v>133</v>
+        <v>2795</v>
       </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="17" t="n">
-        <v>0.12988281</v>
+        <v>2.72949219</v>
       </c>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="inlineStr"/>
@@ -4684,12 +4005,12 @@
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n">
-        <v>133</v>
+        <v>7852</v>
       </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="n"/>
       <c r="L22" s="17" t="n">
-        <v>0.12988281</v>
+        <v>7.66796875</v>
       </c>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="inlineStr"/>
@@ -5138,7 +4459,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -5156,13 +4477,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>128</v>
+        <v>320</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -5234,12 +4555,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3108</v>
+        <v>16064</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>3.03515625</v>
+        <v>15.6875</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -5275,19 +4596,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>344</v>
+        <v>712</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>688</v>
+        <v>1424</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.5859375</v>
@@ -5341,12 +4662,12 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>146</v>
+        <v>3074</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.28515625</v>
+        <v>6.00390625</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
@@ -5438,19 +4759,19 @@
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>344</v>
+        <v>712</v>
       </c>
       <c r="I18" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J18" s="16" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="K18" s="16" t="n">
-        <v>344</v>
+        <v>712</v>
       </c>
       <c r="L18" s="17" t="n">
         <v>0.29296875</v>
@@ -5504,12 +4825,12 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
       <c r="I20" s="16" t="n">
-        <v>146</v>
+        <v>3074</v>
       </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="17" t="n">
-        <v>0.14257812</v>
+        <v>3.00195312</v>
       </c>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="inlineStr"/>
@@ -5551,12 +4872,12 @@
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n">
-        <v>146</v>
+        <v>8638</v>
       </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="n"/>
       <c r="L22" s="17" t="n">
-        <v>0.14257812</v>
+        <v>8.43554688</v>
       </c>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="inlineStr"/>
@@ -5767,7 +5088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O29"/>
+  <dimension ref="B1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5790,7 +5111,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>DR Environment On Premise</t>
+          <t>PRE-PROD Environment On Premise</t>
         </is>
       </c>
     </row>
@@ -6005,7 +5326,7 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
@@ -6023,13 +5344,13 @@
         <v>256</v>
       </c>
       <c r="J7" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="K7" s="19" t="n">
-        <v>128</v>
-      </c>
       <c r="L7" s="20" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
@@ -6056,7 +5377,7 @@
         </is>
       </c>
       <c r="D9" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
@@ -6074,13 +5395,13 @@
         <v>256</v>
       </c>
       <c r="J9" s="16" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K9" s="16" t="n">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="L9" s="17" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="M9" s="16" t="n"/>
       <c r="N9" s="16" t="inlineStr"/>
@@ -6101,12 +5422,12 @@
       <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n">
-        <v>3108</v>
+        <v>9792</v>
       </c>
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="n"/>
       <c r="L10" s="20" t="n">
-        <v>3.03515625</v>
+        <v>9.5625</v>
       </c>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
@@ -6133,7 +5454,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
@@ -6142,22 +5463,22 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>344</v>
+        <v>488</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>688</v>
+        <v>488</v>
       </c>
       <c r="L12" s="17" t="n">
-        <v>0.5859375</v>
+        <v>0.29296875</v>
       </c>
       <c r="M12" s="16" t="n"/>
       <c r="N12" s="16" t="inlineStr"/>
@@ -6171,7 +5492,7 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
@@ -6197,7 +5518,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
@@ -6208,80 +5529,71 @@
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="16" t="n">
-        <v>146</v>
+        <v>2100</v>
       </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="17" t="n">
-        <v>0.28515625</v>
+        <v>2.05078125</v>
       </c>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="inlineStr"/>
       <c r="O14" s="16" t="n"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>RAC - Active/Active</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>20K IOPS</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>As per current archival database size</t>
-        </is>
-      </c>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="19" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J15" s="19" t="n"/>
-      <c r="K15" s="19" t="n"/>
-      <c r="L15" s="20" t="n">
-        <v>4.8828125</v>
-      </c>
-      <c r="M15" s="19" t="n"/>
-      <c r="N15" s="19" t="inlineStr"/>
-      <c r="O15" s="19" t="n"/>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="M15" s="14" t="n"/>
+      <c r="N15" s="14" t="n"/>
+      <c r="O15" s="14" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="B16" s="15" t="n"/>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Dataguard</t>
+          <t>S3 Storage</t>
         </is>
       </c>
       <c r="D16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="16" t="inlineStr"/>
-      <c r="F16" s="16" t="inlineStr"/>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>To be consumed from main NFS storage</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Will be based on the number of documents provided, Considering per document size per Service Request of 512KB Each.</t>
+        </is>
+      </c>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
+      <c r="I16" s="16" t="n">
+        <v>5900</v>
+      </c>
       <c r="J16" s="16" t="n"/>
       <c r="K16" s="16" t="n"/>
-      <c r="L16" s="16" t="n"/>
+      <c r="L16" s="17" t="n">
+        <v>5.76171875</v>
+      </c>
       <c r="M16" s="16" t="n"/>
       <c r="N16" s="16" t="inlineStr"/>
       <c r="O16" s="16" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Oracle Database - Reporting</t>
+          <t>Infrastructure &amp; Monitoring</t>
         </is>
       </c>
       <c r="M17" s="14" t="n"/>
@@ -6289,339 +5601,158 @@
       <c r="O17" s="14" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>OEL/RHEL</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr"/>
-      <c r="G18" s="16" t="n">
-        <v>21</v>
-      </c>
-      <c r="H18" s="16" t="n">
-        <v>344</v>
-      </c>
-      <c r="I18" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="J18" s="16" t="n">
-        <v>21</v>
-      </c>
-      <c r="K18" s="16" t="n">
-        <v>344</v>
-      </c>
-      <c r="L18" s="17" t="n">
-        <v>0.29296875</v>
-      </c>
-      <c r="M18" s="16" t="n"/>
-      <c r="N18" s="16" t="inlineStr"/>
-      <c r="O18" s="16" t="n"/>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>SSL</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Provided by Bank</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="19" t="inlineStr"/>
+      <c r="O18" s="19" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>Oracle License</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr"/>
-      <c r="G19" s="19" t="n"/>
-      <c r="H19" s="19" t="n"/>
-      <c r="I19" s="19" t="n"/>
-      <c r="J19" s="19" t="n"/>
-      <c r="K19" s="19" t="n"/>
-      <c r="L19" s="19" t="n"/>
-      <c r="M19" s="19" t="n"/>
-      <c r="N19" s="19" t="inlineStr"/>
-      <c r="O19" s="19" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Image Registry</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>For Containers docker images</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n">
+        <v>1024</v>
+      </c>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="16" t="n"/>
+      <c r="N19" s="16" t="inlineStr"/>
+      <c r="O19" s="16" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Storage: SAN</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>20K IOPS</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n">
-        <v>146</v>
-      </c>
-      <c r="J20" s="16" t="n"/>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="17" t="n">
-        <v>0.14257812</v>
-      </c>
-      <c r="M20" s="16" t="n"/>
-      <c r="N20" s="16" t="inlineStr"/>
-      <c r="O20" s="16" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="M21" s="14" t="n"/>
-      <c r="N21" s="14" t="n"/>
-      <c r="O21" s="14" t="n"/>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Web Application Firewall (WAF)</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="19" t="inlineStr"/>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>As per banks security policy.</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19" t="n"/>
+      <c r="I20" s="19" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="19" t="n"/>
+      <c r="M20" s="19" t="n"/>
+      <c r="N20" s="19" t="inlineStr"/>
+      <c r="O20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Bastion Host</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="16" t="inlineStr"/>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>As per banks policy.</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="I21" s="16" t="n">
+        <v>256</v>
+      </c>
+      <c r="J21" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="L21" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M21" s="16" t="n"/>
+      <c r="N21" s="16" t="inlineStr"/>
+      <c r="O21" s="16" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>S3 Storage</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>To be consumed from main NFS storage</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>Will be based on the number of documents provided, Considering per document size per Service Request of 512KB Each.</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="16" t="n"/>
-      <c r="I22" s="16" t="n">
-        <v>146</v>
-      </c>
-      <c r="J22" s="16" t="n"/>
-      <c r="K22" s="16" t="n"/>
-      <c r="L22" s="17" t="n">
-        <v>0.14257812</v>
-      </c>
-      <c r="M22" s="16" t="n"/>
-      <c r="N22" s="16" t="inlineStr"/>
-      <c r="O22" s="16" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Infrastructure &amp; Monitoring</t>
-        </is>
-      </c>
-      <c r="M23" s="14" t="n"/>
-      <c r="N23" s="14" t="n"/>
-      <c r="O23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>SSL</t>
-        </is>
-      </c>
-      <c r="D24" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>Provided by Bank</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr"/>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="19" t="n"/>
-      <c r="I24" s="19" t="n"/>
-      <c r="J24" s="19" t="n"/>
-      <c r="K24" s="19" t="n"/>
-      <c r="L24" s="19" t="n"/>
-      <c r="M24" s="19" t="n"/>
-      <c r="N24" s="19" t="inlineStr"/>
-      <c r="O24" s="19" t="n"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Image Registry</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>For Containers docker images</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
-      <c r="I25" s="16" t="n">
-        <v>1024</v>
-      </c>
-      <c r="J25" s="16" t="n"/>
-      <c r="K25" s="16" t="n"/>
-      <c r="L25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" s="16" t="n"/>
-      <c r="N25" s="16" t="inlineStr"/>
-      <c r="O25" s="16" t="n"/>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>Web Application Firewall (WAF)</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="19" t="inlineStr"/>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>As per banks security policy.</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="19" t="n"/>
-      <c r="I26" s="19" t="n"/>
-      <c r="J26" s="19" t="n"/>
-      <c r="K26" s="19" t="n"/>
-      <c r="L26" s="19" t="n"/>
-      <c r="M26" s="19" t="n"/>
-      <c r="N26" s="19" t="inlineStr"/>
-      <c r="O26" s="19" t="n"/>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Bastion Host</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="16" t="inlineStr"/>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>As per banks policy.</t>
-        </is>
-      </c>
-      <c r="G27" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="I27" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J27" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K27" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="L27" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M27" s="16" t="n"/>
-      <c r="N27" s="16" t="inlineStr"/>
-      <c r="O27" s="16" t="n"/>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Email Service</t>
         </is>
       </c>
-      <c r="D28" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="19" t="inlineStr">
+      <c r="D22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>Two million mails/month</t>
         </is>
       </c>
-      <c r="F28" s="19" t="inlineStr"/>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
-      <c r="I28" s="19" t="n"/>
-      <c r="J28" s="19" t="n"/>
-      <c r="K28" s="19" t="n"/>
-      <c r="L28" s="19" t="n"/>
-      <c r="M28" s="19" t="n"/>
-      <c r="N28" s="19" t="inlineStr"/>
-      <c r="O28" s="19" t="n"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>Back Up - DB</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="19" t="inlineStr">
-        <is>
-          <t>As per banks retention policy. Backup solution can be used.</t>
-        </is>
-      </c>
-      <c r="F29" s="19" t="inlineStr"/>
-      <c r="G29" s="19" t="n"/>
-      <c r="H29" s="19" t="n"/>
-      <c r="I29" s="19" t="n"/>
-      <c r="J29" s="19" t="n"/>
-      <c r="K29" s="19" t="n"/>
-      <c r="L29" s="19" t="n"/>
-      <c r="M29" s="19" t="n"/>
-      <c r="N29" s="19" t="inlineStr"/>
-      <c r="O29" s="19" t="n"/>
+      <c r="F22" s="19" t="inlineStr"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
+      <c r="I22" s="19" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="inlineStr"/>
+      <c r="O22" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="B1:N1"/>
-    <mergeCell ref="C23:O23"/>
     <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C3:O3"/>
     <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C21:O21"/>
+    <mergeCell ref="C15:O15"/>
     <mergeCell ref="C11:O11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6657,684 +5788,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>PRE-PROD Environment On Premise</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>S.N.</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>Services/Instances</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Nodes</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Instance Type</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-CPU cores</t>
-        </is>
-      </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-RAM</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>Per Node
-Storage (GB)</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-CPU cores</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-RAM
-(GB)</t>
-        </is>
-      </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>Total
-Storage
-(TB)</t>
-        </is>
-      </c>
-      <c r="M2" s="13" t="n"/>
-      <c r="N2" s="13" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="O2" s="13" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="B3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Kubeadm Cluster</t>
-        </is>
-      </c>
-      <c r="M3" s="14" t="n"/>
-      <c r="N3" s="14" t="n"/>
-      <c r="O3" s="14" t="n"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Bootstrap machine</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>Kubeadm vendor to confirm on sizing.</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I4" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J4" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="L4" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M4" s="16" t="n"/>
-      <c r="N4" s="16" t="inlineStr"/>
-      <c r="O4" s="16" t="n"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>Bastion Host</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="inlineStr"/>
-      <c r="G5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>256</v>
-      </c>
-      <c r="J5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M5" s="19" t="n"/>
-      <c r="N5" s="19" t="inlineStr"/>
-      <c r="O5" s="19" t="n"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Master Nodes</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr"/>
-      <c r="G6" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J6" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="L6" s="17" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="M6" s="16" t="n"/>
-      <c r="N6" s="16" t="inlineStr"/>
-      <c r="O6" s="16" t="n"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Linux Worker Nodes (BUSINESSNEXT)</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F7" s="19" t="inlineStr"/>
-      <c r="G7" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>256</v>
-      </c>
-      <c r="J7" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="L7" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M7" s="19" t="n"/>
-      <c r="N7" s="19" t="inlineStr"/>
-      <c r="O7" s="19" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Operational Services</t>
-        </is>
-      </c>
-      <c r="M8" s="14" t="n"/>
-      <c r="N8" s="14" t="n"/>
-      <c r="O8" s="14" t="n"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Infra Nodes (Grafana &amp; Prometheus, EFK, Redis)</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Compute Intensive</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr"/>
-      <c r="G9" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J9" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="K9" s="16" t="n">
-        <v>64</v>
-      </c>
-      <c r="L9" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M9" s="16" t="n"/>
-      <c r="N9" s="16" t="inlineStr"/>
-      <c r="O9" s="16" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>NFS Storage</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr"/>
-      <c r="F10" s="19" t="inlineStr"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n">
-        <v>1992</v>
-      </c>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="20" t="n">
-        <v>1.9453125</v>
-      </c>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="19" t="inlineStr"/>
-      <c r="O10" s="19" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Oracle Database</t>
-        </is>
-      </c>
-      <c r="M11" s="14" t="n"/>
-      <c r="N11" s="14" t="n"/>
-      <c r="O11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>OEL/RHEL</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="H12" s="16" t="n">
-        <v>240</v>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="J12" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="K12" s="16" t="n">
-        <v>240</v>
-      </c>
-      <c r="L12" s="17" t="n">
-        <v>0.29296875</v>
-      </c>
-      <c r="M12" s="16" t="n"/>
-      <c r="N12" s="16" t="inlineStr"/>
-      <c r="O12" s="16" t="n"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>Oracle License</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>Memory Intensive</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="inlineStr"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="19" t="n"/>
-      <c r="L13" s="19" t="n"/>
-      <c r="M13" s="19" t="n"/>
-      <c r="N13" s="19" t="inlineStr"/>
-      <c r="O13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Storage: SAN</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>20K IOPS</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr"/>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="J14" s="16" t="n"/>
-      <c r="K14" s="16" t="n"/>
-      <c r="L14" s="17" t="n">
-        <v>0.09765625</v>
-      </c>
-      <c r="M14" s="16" t="n"/>
-      <c r="N14" s="16" t="inlineStr"/>
-      <c r="O14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="n"/>
-      <c r="N15" s="14" t="n"/>
-      <c r="O15" s="14" t="n"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>S3 Storage</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>To be consumed from main NFS storage</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>Will be based on the number of documents provided, Considering per document size per Service Request of 512KB Each.</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="17" t="n">
-        <v>0.09765625</v>
-      </c>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="16" t="inlineStr"/>
-      <c r="O16" s="16" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Infrastructure &amp; Monitoring</t>
-        </is>
-      </c>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="14" t="n"/>
-      <c r="O17" s="14" t="n"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>SSL</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>Provided by Bank</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr"/>
-      <c r="G18" s="19" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="19" t="n"/>
-      <c r="J18" s="19" t="n"/>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="19" t="n"/>
-      <c r="M18" s="19" t="n"/>
-      <c r="N18" s="19" t="inlineStr"/>
-      <c r="O18" s="19" t="n"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Image Registry</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>For Containers docker images</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n">
-        <v>1024</v>
-      </c>
-      <c r="J19" s="16" t="n"/>
-      <c r="K19" s="16" t="n"/>
-      <c r="L19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="inlineStr"/>
-      <c r="O19" s="16" t="n"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>Web Application Firewall (WAF)</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="19" t="inlineStr"/>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>As per banks security policy.</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="19" t="n"/>
-      <c r="N20" s="19" t="inlineStr"/>
-      <c r="O20" s="19" t="n"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Bastion Host</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="16" t="inlineStr"/>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>As per banks policy.</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="I21" s="16" t="n">
-        <v>256</v>
-      </c>
-      <c r="J21" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="L21" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="16" t="inlineStr"/>
-      <c r="O21" s="16" t="n"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Email Service</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>Two million mails/month</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="19" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
-      <c r="M22" s="19" t="n"/>
-      <c r="N22" s="19" t="inlineStr"/>
-      <c r="O22" s="19" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C15:O15"/>
-    <mergeCell ref="C11:O11"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:O22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="4" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
-    <col width="4" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>UAT Environment On Premise</t>
+          <t>SIT Environment On Premise</t>
         </is>
       </c>
     </row>
@@ -7686,19 +6140,19 @@
       </c>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>240</v>
+        <v>488</v>
       </c>
       <c r="I12" s="16" t="n">
         <v>300</v>
       </c>
       <c r="J12" s="16" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>240</v>
+        <v>488</v>
       </c>
       <c r="L12" s="17" t="n">
         <v>0.29296875</v>

</xml_diff>